<commit_message>
Cleans up the nba data sheet
</commit_message>
<xml_diff>
--- a/NBACareerPredictor/data/NBAProspects2026.xlsx
+++ b/NBACareerPredictor/data/NBAProspects2026.xlsx
@@ -5,18 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/A88D152AB49A4EE2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a88d152ab49a4ee2/Documents/DataScienceProjects/NBACareerPredictor/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="804" documentId="8_{40287C8F-6A9D-4D9F-A391-776DE7561C97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED2CC3D3-DEF0-4A65-B53D-B1B49346DD99}"/>
+  <xr:revisionPtr revIDLastSave="806" documentId="8_{40287C8F-6A9D-4D9F-A391-776DE7561C97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF794BC6-70E8-4E6B-A95B-2C866438D8B5}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{E99D141E-76A2-4C01-86EB-E886F75FFC28}"/>
+    <workbookView minimized="1" xWindow="8004" yWindow="7680" windowWidth="7500" windowHeight="6000" xr2:uid="{E99D141E-76A2-4C01-86EB-E886F75FFC28}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -126,12 +125,6 @@
     <t>PTS</t>
   </si>
   <si>
-    <t>ORtg</t>
-  </si>
-  <si>
-    <t>DRtg</t>
-  </si>
-  <si>
     <t>BYU</t>
   </si>
   <si>
@@ -544,6 +537,12 @@
   </si>
   <si>
     <t>Auburn</t>
+  </si>
+  <si>
+    <t>ORTG</t>
+  </si>
+  <si>
+    <t>DRTG</t>
   </si>
 </sst>
 </file>
@@ -586,12 +585,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -931,7 +929,7 @@
   <sheetData>
     <row r="1" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1021,87 +1019,87 @@
         <v>28</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>29</v>
+        <v>167</v>
       </c>
       <c r="AF1" t="s">
-        <v>30</v>
+        <v>168</v>
       </c>
       <c r="AG1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AI1" t="s">
         <v>35</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AJ1" t="s">
         <v>36</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AK1" t="s">
         <v>37</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AL1" t="s">
         <v>38</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AM1" t="s">
         <v>39</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AN1" t="s">
         <v>40</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AO1" t="s">
         <v>41</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AP1" t="s">
         <v>42</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AQ1" t="s">
         <v>43</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AR1" t="s">
         <v>44</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AS1" t="s">
         <v>45</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AT1" t="s">
         <v>46</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AU1" t="s">
         <v>47</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AV1" t="s">
         <v>48</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AW1" t="s">
         <v>49</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AX1" t="s">
         <v>50</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AY1" t="s">
         <v>51</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="AZ1" t="s">
         <v>52</v>
-      </c>
-      <c r="AY1" t="s">
-        <v>53</v>
-      </c>
-      <c r="AZ1" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" t="s">
         <v>31</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>32</v>
-      </c>
-      <c r="D2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E2" t="s">
-        <v>34</v>
       </c>
       <c r="F2">
         <v>35</v>
@@ -1247,16 +1245,16 @@
     </row>
     <row r="3" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E3" t="s">
         <v>4</v>
@@ -1405,19 +1403,19 @@
     </row>
     <row r="4" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F4">
         <v>38</v>
@@ -1563,19 +1561,19 @@
     </row>
     <row r="5" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C5" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F5">
         <v>24</v>
@@ -1721,16 +1719,16 @@
     </row>
     <row r="6" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C6" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E6" t="s">
         <v>4</v>
@@ -1879,16 +1877,16 @@
     </row>
     <row r="7" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C7" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E7" t="s">
         <v>4</v>
@@ -2037,16 +2035,16 @@
     </row>
     <row r="8" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C8" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D8" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E8" t="s">
         <v>4</v>
@@ -2195,19 +2193,19 @@
     </row>
     <row r="9" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C9" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E9" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F9">
         <v>35</v>
@@ -2353,16 +2351,16 @@
     </row>
     <row r="10" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C10" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D10" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E10" t="s">
         <v>4</v>
@@ -2511,16 +2509,16 @@
     </row>
     <row r="11" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C11" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D11" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E11" t="s">
         <v>4</v>
@@ -2669,19 +2667,19 @@
     </row>
     <row r="12" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C12" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D12" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E12" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F12">
         <v>31</v>
@@ -2827,19 +2825,19 @@
     </row>
     <row r="13" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C13" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D13" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E13" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F13">
         <v>40</v>
@@ -2985,19 +2983,19 @@
     </row>
     <row r="14" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C14" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D14" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E14" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F14">
         <v>34</v>
@@ -3143,19 +3141,19 @@
     </row>
     <row r="15" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C15" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D15" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E15" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F15">
         <v>40</v>
@@ -3301,19 +3299,19 @@
     </row>
     <row r="16" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D16" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E16" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F16">
         <v>30</v>
@@ -3459,16 +3457,16 @@
     </row>
     <row r="17" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C17" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D17" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E17" t="s">
         <v>4</v>
@@ -3617,16 +3615,16 @@
     </row>
     <row r="18" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C18" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D18" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E18" t="s">
         <v>4</v>
@@ -3775,19 +3773,19 @@
     </row>
     <row r="19" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C19" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D19" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E19" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F19">
         <v>37</v>
@@ -3933,16 +3931,16 @@
     </row>
     <row r="20" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C20" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D20" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E20" t="s">
         <v>4</v>
@@ -4091,19 +4089,19 @@
     </row>
     <row r="21" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C21" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D21" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E21" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F21">
         <v>4</v>
@@ -4249,16 +4247,16 @@
     </row>
     <row r="22" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C22" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D22" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E22" t="s">
         <v>4</v>
@@ -4407,19 +4405,19 @@
     </row>
     <row r="23" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C23" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D23" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E23" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F23">
         <v>35</v>
@@ -4565,16 +4563,16 @@
     </row>
     <row r="24" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D24" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E24" t="s">
         <v>4</v>
@@ -4723,16 +4721,16 @@
     </row>
     <row r="25" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C25" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D25" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E25" t="s">
         <v>4</v>
@@ -4881,19 +4879,19 @@
     </row>
     <row r="26" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C26" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D26" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E26" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F26">
         <v>36</v>
@@ -5039,19 +5037,19 @@
     </row>
     <row r="27" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C27" t="s">
+        <v>30</v>
+      </c>
+      <c r="D27" t="s">
+        <v>31</v>
+      </c>
+      <c r="E27" t="s">
         <v>32</v>
-      </c>
-      <c r="D27" t="s">
-        <v>33</v>
-      </c>
-      <c r="E27" t="s">
-        <v>34</v>
       </c>
       <c r="F27">
         <v>36</v>
@@ -5197,19 +5195,19 @@
     </row>
     <row r="28" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C28" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D28" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E28" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F28">
         <v>40</v>
@@ -5355,16 +5353,16 @@
     </row>
     <row r="29" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D29" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E29" t="s">
         <v>4</v>
@@ -5513,16 +5511,16 @@
     </row>
     <row r="30" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C30" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D30" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E30" t="s">
         <v>4</v>
@@ -5671,19 +5669,19 @@
     </row>
     <row r="31" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C31" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D31" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E31" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F31">
         <v>31</v>
@@ -5829,19 +5827,19 @@
     </row>
     <row r="32" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C32" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D32" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E32" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F32">
         <v>37</v>
@@ -5987,19 +5985,19 @@
     </row>
     <row r="33" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C33" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D33" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E33" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F33">
         <v>40</v>
@@ -6145,19 +6143,19 @@
     </row>
     <row r="34" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C34" t="s">
+        <v>30</v>
+      </c>
+      <c r="D34" t="s">
+        <v>108</v>
+      </c>
+      <c r="E34" t="s">
         <v>32</v>
-      </c>
-      <c r="D34" t="s">
-        <v>110</v>
-      </c>
-      <c r="E34" t="s">
-        <v>34</v>
       </c>
       <c r="F34">
         <v>35</v>
@@ -6303,19 +6301,19 @@
     </row>
     <row r="35" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C35" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D35" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E35" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F35">
         <v>16</v>
@@ -6461,19 +6459,19 @@
     </row>
     <row r="36" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C36" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D36" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E36" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F36">
         <v>35</v>
@@ -6619,19 +6617,19 @@
     </row>
     <row r="37" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C37" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D37" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E37" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F37">
         <v>28</v>
@@ -6777,16 +6775,16 @@
     </row>
     <row r="38" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C38" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D38" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E38" t="s">
         <v>4</v>
@@ -6935,19 +6933,19 @@
     </row>
     <row r="39" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C39" t="s">
+        <v>30</v>
+      </c>
+      <c r="D39" t="s">
+        <v>108</v>
+      </c>
+      <c r="E39" t="s">
         <v>32</v>
-      </c>
-      <c r="D39" t="s">
-        <v>110</v>
-      </c>
-      <c r="E39" t="s">
-        <v>34</v>
       </c>
       <c r="F39">
         <v>31</v>
@@ -7093,16 +7091,16 @@
     </row>
     <row r="40" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C40" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D40" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E40" t="s">
         <v>4</v>
@@ -7146,7 +7144,7 @@
       <c r="R40">
         <v>0.52300000000000002</v>
       </c>
-      <c r="S40" s="2">
+      <c r="S40">
         <v>1.2</v>
       </c>
       <c r="T40">
@@ -7251,16 +7249,16 @@
     </row>
     <row r="41" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C41" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D41" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E41" t="s">
         <v>4</v>
@@ -7409,16 +7407,16 @@
     </row>
     <row r="42" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B42" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C42" t="s">
+        <v>30</v>
+      </c>
+      <c r="D42" t="s">
         <v>108</v>
-      </c>
-      <c r="C42" t="s">
-        <v>32</v>
-      </c>
-      <c r="D42" t="s">
-        <v>110</v>
       </c>
       <c r="E42" t="s">
         <v>4</v>
@@ -7567,16 +7565,16 @@
     </row>
     <row r="43" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C43" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D43" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E43" t="s">
         <v>4</v>
@@ -7725,19 +7723,19 @@
     </row>
     <row r="44" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C44" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D44" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E44" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F44">
         <v>37</v>
@@ -7883,19 +7881,19 @@
     </row>
     <row r="45" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C45" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D45" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E45" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F45">
         <v>36</v>
@@ -8041,16 +8039,16 @@
     </row>
     <row r="46" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C46" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D46" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E46" t="s">
         <v>4</v>
@@ -8199,16 +8197,16 @@
     </row>
     <row r="47" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C47" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D47" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E47" t="s">
         <v>4</v>
@@ -8357,19 +8355,19 @@
     </row>
     <row r="48" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C48" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D48" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E48" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F48">
         <v>35</v>
@@ -8515,19 +8513,19 @@
     </row>
     <row r="49" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C49" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D49" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E49" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F49">
         <v>34</v>
@@ -8673,19 +8671,19 @@
     </row>
     <row r="50" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C50" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D50" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E50" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F50">
         <v>37</v>
@@ -8831,19 +8829,19 @@
     </row>
     <row r="51" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C51" t="s">
+        <v>30</v>
+      </c>
+      <c r="D51" t="s">
+        <v>110</v>
+      </c>
+      <c r="E51" t="s">
         <v>32</v>
-      </c>
-      <c r="D51" t="s">
-        <v>112</v>
-      </c>
-      <c r="E51" t="s">
-        <v>34</v>
       </c>
       <c r="F51">
         <v>39</v>
@@ -8989,19 +8987,19 @@
     </row>
     <row r="52" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C52" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D52" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E52" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F52">
         <v>36</v>
@@ -9147,19 +9145,19 @@
     </row>
     <row r="53" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C53" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D53" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E53" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F53">
         <v>30</v>
@@ -9305,16 +9303,16 @@
     </row>
     <row r="54" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C54" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D54" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E54" t="s">
         <v>4</v>
@@ -9463,19 +9461,19 @@
     </row>
     <row r="55" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C55" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D55" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E55" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F55">
         <v>33</v>
@@ -9621,19 +9619,19 @@
     </row>
     <row r="56" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C56" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D56" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E56" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F56">
         <v>38</v>
@@ -9779,16 +9777,16 @@
     </row>
     <row r="57" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C57" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D57" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E57" t="s">
         <v>4</v>
@@ -9937,19 +9935,19 @@
     </row>
     <row r="58" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C58" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D58" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E58" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F58">
         <v>31</v>
@@ -10095,16 +10093,16 @@
     </row>
     <row r="59" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C59" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D59" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E59" t="s">
         <v>4</v>
@@ -10253,16 +10251,16 @@
     </row>
     <row r="60" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C60" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D60" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E60" t="s">
         <v>4</v>
@@ -10411,19 +10409,19 @@
     </row>
     <row r="61" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C61" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D61" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E61" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F61">
         <v>25</v>
@@ -10569,19 +10567,19 @@
     </row>
     <row r="62" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C62" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D62" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E62" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F62">
         <v>39</v>
@@ -10724,16 +10722,16 @@
     </row>
     <row r="63" spans="1:52" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C63" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D63" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E63" t="s">
         <v>4</v>

</xml_diff>